<commit_message>
v2.5: propose large N-to-1 splits — equal instalments and round-denomination batches
A 13,000,000 SAP posting paid by the bank as 10 x 1,000,000 + 6 x 500,000
was invisible to the split search (DFS capped at 6 members) and to 1-to-1
line matching. When the bounded DFS finds nothing, two cheap strategies now
run with a 60-member cap: greedy composition from the largest available
denominations downwards, then k equal instalments (exact cents division).
Both respect the same-sign, date-window and prefix filters, and results
remain user-approved proposals.

Validated on the real BOC files (user's settings): 13M = 10x1M + 6x500k
diff 0.00, 11M = 22x500k diff 0.00, 6,216,168.10 payroll = 2 lines diff
0.00. Fixture adds a 13 x 1M batch; all suites green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNPLbA1ZQMqWR2Ur5MwfPL
</commit_message>
<xml_diff>
--- a/recon-tool/samples/split_A.xlsx
+++ b/recon-tool/samples/split_A.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,49 +415,63 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>INV-500</v>
+        <v>INV-13M</v>
       </c>
       <c r="B2" t="str">
-        <v>01/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C2" t="str">
-        <v>Προμηθευτής ΑΛΦΑ</v>
+        <v>Μεταφορά σε λογαριασμό εξόδων</v>
       </c>
       <c r="D2">
-        <v>500</v>
+        <v>13000000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>INV-300</v>
+        <v>INV-500</v>
       </c>
       <c r="B3" t="str">
-        <v>05/03/2026</v>
+        <v>01/03/2026</v>
       </c>
       <c r="C3" t="str">
-        <v>Προμηθευτής ΒΗΤΑ</v>
+        <v>Προμηθευτής ΑΛΦΑ</v>
       </c>
       <c r="D3">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>INV-300</v>
+      </c>
+      <c r="B4" t="str">
+        <v>05/03/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Προμηθευτής ΒΗΤΑ</v>
+      </c>
+      <c r="D4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>INV-250</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>10/03/2026</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C5" t="str">
         <v>Προμηθευτής ΓΑΜΑ</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <v>250.01</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>